<commit_message>
#12 Update BOM and Centroid file Create Also.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/JLCPCB_BOM.xlsx
+++ b/Deliverables/BOM/JLCPCB_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ezlo-switchbox\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1945F7-54F9-45A3-A0D9-0FA7ABE1048B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8007C3C-9F0E-49AA-8B58-25B1804F79B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -262,9 +262,6 @@
     <t>RES-0603</t>
   </si>
   <si>
-    <t>Res-0402x4</t>
-  </si>
-  <si>
     <t>Res-0402</t>
   </si>
   <si>
@@ -337,9 +334,6 @@
     <t>C105433</t>
   </si>
   <si>
-    <t>C162973</t>
-  </si>
-  <si>
     <t>C413056</t>
   </si>
   <si>
@@ -386,6 +380,12 @@
   </si>
   <si>
     <t>C131394</t>
+  </si>
+  <si>
+    <t>C12018</t>
+  </si>
+  <si>
+    <t>Res-0603x4</t>
   </si>
 </sst>
 </file>
@@ -448,7 +448,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -530,11 +530,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -562,6 +584,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -870,7 +898,7 @@
         <v>66</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -884,7 +912,7 @@
         <v>67</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -898,7 +926,7 @@
         <v>68</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -912,7 +940,7 @@
         <v>69</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -926,7 +954,7 @@
         <v>69</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -940,7 +968,7 @@
         <v>70</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -954,7 +982,7 @@
         <v>68</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -968,7 +996,7 @@
         <v>68</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -982,7 +1010,7 @@
         <v>68</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -996,7 +1024,7 @@
         <v>71</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1010,7 +1038,7 @@
         <v>72</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1024,7 +1052,7 @@
         <v>73</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1038,7 +1066,7 @@
         <v>11</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1052,7 +1080,7 @@
         <v>74</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1066,7 +1094,7 @@
         <v>13</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1080,7 +1108,7 @@
         <v>75</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1094,7 +1122,7 @@
         <v>15</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1108,7 +1136,7 @@
         <v>76</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1122,7 +1150,7 @@
         <v>77</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1136,7 +1164,7 @@
         <v>78</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1150,7 +1178,7 @@
         <v>78</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1158,13 +1186,13 @@
         <v>20</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>79</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1175,10 +1203,10 @@
         <v>54</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>80</v>
+        <v>121</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1189,10 +1217,10 @@
         <v>55</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1203,10 +1231,10 @@
         <v>56</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1217,10 +1245,10 @@
         <v>57</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1231,10 +1259,10 @@
         <v>58</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1245,10 +1273,10 @@
         <v>59</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1262,7 +1290,7 @@
         <v>27</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1273,10 +1301,10 @@
         <v>61</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1287,10 +1315,10 @@
         <v>62</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1301,10 +1329,10 @@
         <v>63</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1315,24 +1343,24 @@
         <v>64</v>
       </c>
       <c r="C33" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="D33" s="6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>114</v>
+      <c r="D34" s="10" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
switchbox centroid file corrected
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/JLCPCB_BOM.xlsx
+++ b/Deliverables/BOM/JLCPCB_BOM.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ezlo-switchbox\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ezlo-switchbox\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8007C3C-9F0E-49AA-8B58-25B1804F79B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="116">
   <si>
     <t>Comment</t>
   </si>
@@ -40,9 +39,6 @@
     <t>4.7nF</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>4.7uF</t>
   </si>
   <si>
@@ -73,9 +69,6 @@
     <t>Green</t>
   </si>
   <si>
-    <t>TEST POINT</t>
-  </si>
-  <si>
     <t>FDN306P</t>
   </si>
   <si>
@@ -139,9 +132,6 @@
     <t>C10</t>
   </si>
   <si>
-    <t>C11, C12</t>
-  </si>
-  <si>
     <t>C13</t>
   </si>
   <si>
@@ -175,9 +165,6 @@
     <t>LED1, LED2, LED3, LED4, LED5, LED6, LED7, LED8, LED9, LED10</t>
   </si>
   <si>
-    <t>P2, P3, P14, P15</t>
-  </si>
-  <si>
     <t>Q2</t>
   </si>
   <si>
@@ -253,9 +240,6 @@
     <t>LED-0402</t>
   </si>
   <si>
-    <t>Test-point</t>
-  </si>
-  <si>
     <t>SOT-23</t>
   </si>
   <si>
@@ -365,9 +349,6 @@
   </si>
   <si>
     <t>C96446</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>C105873</t>
@@ -391,7 +372,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -876,9 +857,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -892,13 +873,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -906,13 +887,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -920,13 +901,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -934,13 +915,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -948,13 +929,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -962,181 +943,181 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C8" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="D13" s="4" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="5" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="7" t="s">
+      <c r="D15" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="D17" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1144,27 +1125,27 @@
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>52</v>
+      <c r="B20" s="8" t="s">
+        <v>108</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>102</v>
+        <v>74</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1172,27 +1153,27 @@
         <v>19</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>113</v>
+      <c r="B22" s="4" t="s">
+        <v>51</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>106</v>
+        <v>75</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1200,13 +1181,13 @@
         <v>21</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>121</v>
+        <v>75</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1214,13 +1195,13 @@
         <v>22</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1228,27 +1209,27 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1256,13 +1237,13 @@
         <v>25</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1270,13 +1251,13 @@
         <v>26</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1284,27 +1265,27 @@
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1312,55 +1293,27 @@
         <v>29</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>112</v>
+      <c r="B32" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>